<commit_message>
Revised database template again
</commit_message>
<xml_diff>
--- a/instance/logsheet_template.xlsx
+++ b/instance/logsheet_template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Rigel\Documents\Disaster_Classification\instance\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F698EA24-3870-4146-B9E9-A8BD992CC95A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C35C1971-DE10-47CB-B29F-8967C59639E1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -203,53 +203,16 @@
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>1684868</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="1073202" cy="914400"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="3" name="Image 2" descr="Picture">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000003000000}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr/>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print"/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr>
-        <a:xfrm>
-          <a:off x="7446331" y="0"/>
-          <a:ext cx="1073202" cy="914400"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>3</xdr:col>
-      <xdr:colOff>1003608</xdr:colOff>
+      <xdr:colOff>767256</xdr:colOff>
       <xdr:row>0</xdr:row>
       <xdr:rowOff>1</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>4</xdr:col>
-      <xdr:colOff>810320</xdr:colOff>
+      <xdr:colOff>706695</xdr:colOff>
       <xdr:row>3</xdr:row>
       <xdr:rowOff>41032</xdr:rowOff>
     </xdr:to>
@@ -267,7 +230,7 @@
         </xdr:cNvPicPr>
       </xdr:nvPicPr>
       <xdr:blipFill rotWithShape="1">
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
           <a:extLst>
             <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
               <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
@@ -281,8 +244,59 @@
       </xdr:blipFill>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="4708100" y="1"/>
-          <a:ext cx="902820" cy="867508"/>
+          <a:off x="4466897" y="1"/>
+          <a:ext cx="1037770" cy="860838"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>19145</xdr:colOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>54430</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>940676</xdr:colOff>
+      <xdr:row>3</xdr:row>
+      <xdr:rowOff>59465</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="4" name="Picture 3">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{A71A8171-D2EB-F1B8-3A68-78DF68C0F4A3}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill rotWithShape="1">
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2" cstate="print">
+          <a:extLst>
+            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
+              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
+            </a:ext>
+          </a:extLst>
+        </a:blip>
+        <a:srcRect l="8869" t="9218" r="8029" b="7446"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="7623379" y="54430"/>
+          <a:ext cx="921531" cy="824842"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>

</xml_diff>